<commit_message>
Updated the issues log and bug tracker
</commit_message>
<xml_diff>
--- a/Lopsided Productions Bug Tracker.xlsx
+++ b/Lopsided Productions Bug Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tdigu\Desktop\Insomniac\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBE716C9-B5C3-44DB-81F0-F83B6D85198C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A867F861-786A-40B5-82FE-E8D96789EF8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-7335" yWindow="-13935" windowWidth="21600" windowHeight="11775" xr2:uid="{E426D4A3-675A-4749-AD97-AF7CA7903CDF}"/>
+    <workbookView xWindow="16395" yWindow="-15720" windowWidth="21600" windowHeight="11775" xr2:uid="{E426D4A3-675A-4749-AD97-AF7CA7903CDF}"/>
   </bookViews>
   <sheets>
     <sheet name="Bug Tracker" sheetId="8" r:id="rId1"/>
@@ -65,7 +65,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="33">
   <si>
     <t>Ref #</t>
   </si>
@@ -123,21 +123,12 @@
     <t>J</t>
   </si>
   <si>
-    <t>In-Progress</t>
-  </si>
-  <si>
     <t>BT002</t>
   </si>
   <si>
     <t>Sleep Button</t>
   </si>
   <si>
-    <t>Click navifgation is off. Change events to Left-down.</t>
-  </si>
-  <si>
-    <t>J,N</t>
-  </si>
-  <si>
     <t>Fixed</t>
   </si>
   <si>
@@ -162,10 +153,19 @@
     <t>T</t>
   </si>
   <si>
-    <t>May not be a design bug.</t>
-  </si>
-  <si>
     <t>Last Update:  5/12/2026</t>
+  </si>
+  <si>
+    <t>Jessica, Tom</t>
+  </si>
+  <si>
+    <t>Click navigation is off. Change events to Left-down.</t>
+  </si>
+  <si>
+    <t>Jessica, Nick</t>
+  </si>
+  <si>
+    <t>Reviewed, not a design bug.</t>
   </si>
 </sst>
 </file>
@@ -952,7 +952,7 @@
     <col min="5" max="5" width="19.88671875" style="14" customWidth="1"/>
     <col min="6" max="6" width="14.33203125" style="13" customWidth="1"/>
     <col min="7" max="7" width="13.44140625" style="13" customWidth="1"/>
-    <col min="8" max="8" width="10.109375" style="13" customWidth="1"/>
+    <col min="8" max="8" width="15.5546875" style="13" bestFit="1" customWidth="1"/>
     <col min="9" max="10" width="13.5546875" style="13" customWidth="1"/>
     <col min="11" max="11" width="53.5546875" style="13" customWidth="1"/>
     <col min="12" max="12" width="34.44140625" style="14" customWidth="1"/>
@@ -976,7 +976,7 @@
     </row>
     <row r="2" spans="2:12" s="3" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="16" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="C2" s="16"/>
       <c r="D2" s="16"/>
@@ -1044,7 +1044,7 @@
         <v>46128</v>
       </c>
       <c r="H4" s="7" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="I4" s="7">
         <v>46135</v>
@@ -1053,19 +1053,19 @@
         <v>46134</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="L4" s="6"/>
     </row>
     <row r="5" spans="2:12" ht="26.4" x14ac:dyDescent="0.25">
       <c r="B5" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C5" s="2" t="s">
-        <v>20</v>
-      </c>
       <c r="D5" s="6" t="s">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="E5" s="4" t="s">
         <v>15</v>
@@ -1077,7 +1077,7 @@
         <v>46128</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="I5" s="7">
         <v>46135</v>
@@ -1086,19 +1086,19 @@
         <v>46134</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="L5" s="6"/>
     </row>
     <row r="6" spans="2:12" ht="26.4" x14ac:dyDescent="0.25">
       <c r="B6" s="2" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="E6" s="4" t="s">
         <v>15</v>
@@ -1110,40 +1110,52 @@
         <v>46134</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="I6" s="7">
         <v>46142</v>
       </c>
-      <c r="J6" s="2"/>
+      <c r="J6" s="7">
+        <v>46142</v>
+      </c>
       <c r="K6" s="2" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="L6" s="6"/>
     </row>
     <row r="7" spans="2:12" ht="26.4" x14ac:dyDescent="0.25">
       <c r="B7" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F7" s="4" t="s">
         <v>27</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="D7" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="E7" s="4"/>
-      <c r="F7" s="4" t="s">
-        <v>30</v>
       </c>
       <c r="G7" s="7">
         <v>46135</v>
       </c>
-      <c r="H7" s="2"/>
-      <c r="I7" s="2"/>
-      <c r="J7" s="2"/>
-      <c r="K7" s="2"/>
+      <c r="H7" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="I7" s="7">
+        <v>46145</v>
+      </c>
+      <c r="J7" s="7">
+        <v>46145</v>
+      </c>
+      <c r="K7" s="2" t="s">
+        <v>20</v>
+      </c>
       <c r="L7" s="6" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="8" spans="2:12" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Updated Risk Log and Bug Tracker for 5/14 individual submission
</commit_message>
<xml_diff>
--- a/Lopsided Productions Bug Tracker.xlsx
+++ b/Lopsided Productions Bug Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tdigu\Desktop\Insomniac\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A867F861-786A-40B5-82FE-E8D96789EF8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F943BC7E-6ADF-4CE5-BDE7-A936F9B64D82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="16395" yWindow="-15720" windowWidth="21600" windowHeight="11775" xr2:uid="{E426D4A3-675A-4749-AD97-AF7CA7903CDF}"/>
+    <workbookView xWindow="16635" yWindow="-14505" windowWidth="26715" windowHeight="11775" xr2:uid="{E426D4A3-675A-4749-AD97-AF7CA7903CDF}"/>
   </bookViews>
   <sheets>
     <sheet name="Bug Tracker" sheetId="8" r:id="rId1"/>
@@ -60,12 +60,37 @@
         </r>
       </text>
     </comment>
+    <comment ref="H3" authorId="0" shapeId="0" xr:uid="{4E8EA435-5370-4189-9DFC-2C75AA45B386}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">Coder / Tester
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
+        </r>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="38">
   <si>
     <t>Ref #</t>
   </si>
@@ -117,12 +142,6 @@
     <t>Med</t>
   </si>
   <si>
-    <t>N</t>
-  </si>
-  <si>
-    <t>J</t>
-  </si>
-  <si>
     <t>BT002</t>
   </si>
   <si>
@@ -150,12 +169,6 @@
     <t>When game is open, the window cannot be resized.</t>
   </si>
   <si>
-    <t>T</t>
-  </si>
-  <si>
-    <t>Last Update:  5/12/2026</t>
-  </si>
-  <si>
     <t>Jessica, Tom</t>
   </si>
   <si>
@@ -166,13 +179,40 @@
   </si>
   <si>
     <t>Reviewed, not a design bug.</t>
+  </si>
+  <si>
+    <t>BT005</t>
+  </si>
+  <si>
+    <t>Level 3 sleep state</t>
+  </si>
+  <si>
+    <t>Level 3 allows for multiple monsters to be active at the same time. Sleep state should not be available when multiple monsters are active.</t>
+  </si>
+  <si>
+    <t>High</t>
+  </si>
+  <si>
+    <t>Jessica</t>
+  </si>
+  <si>
+    <t>Tom</t>
+  </si>
+  <si>
+    <t>Nick</t>
+  </si>
+  <si>
+    <t>In-Progress</t>
+  </si>
+  <si>
+    <t>Will be completed prior to 5/17.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -211,6 +251,23 @@
       <name val="Tahoma"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -233,7 +290,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1">
@@ -275,6 +332,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -954,7 +1014,7 @@
     <col min="7" max="7" width="13.44140625" style="13" customWidth="1"/>
     <col min="8" max="8" width="15.5546875" style="13" bestFit="1" customWidth="1"/>
     <col min="9" max="10" width="13.5546875" style="13" customWidth="1"/>
-    <col min="11" max="11" width="53.5546875" style="13" customWidth="1"/>
+    <col min="11" max="11" width="30.6640625" style="13" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="34.44140625" style="14" customWidth="1"/>
     <col min="13" max="16384" width="9.109375" style="8"/>
   </cols>
@@ -975,8 +1035,8 @@
       <c r="L1" s="15"/>
     </row>
     <row r="2" spans="2:12" s="3" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="16" t="s">
-        <v>28</v>
+      <c r="B2" s="17">
+        <v>46156</v>
       </c>
       <c r="C2" s="16"/>
       <c r="D2" s="16"/>
@@ -1038,13 +1098,13 @@
         <v>15</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>16</v>
+        <v>35</v>
       </c>
       <c r="G4" s="7">
         <v>46128</v>
       </c>
       <c r="H4" s="7" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="I4" s="7">
         <v>46135</v>
@@ -1053,31 +1113,31 @@
         <v>46134</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="L4" s="6"/>
     </row>
     <row r="5" spans="2:12" ht="26.4" x14ac:dyDescent="0.25">
       <c r="B5" s="2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="E5" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>16</v>
+        <v>35</v>
       </c>
       <c r="G5" s="7">
         <v>46128</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="I5" s="7">
         <v>46135</v>
@@ -1086,31 +1146,31 @@
         <v>46134</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="L5" s="6"/>
     </row>
     <row r="6" spans="2:12" ht="26.4" x14ac:dyDescent="0.25">
       <c r="B6" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D6" s="6" t="s">
         <v>21</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>23</v>
       </c>
       <c r="E6" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="G6" s="7">
         <v>46134</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="I6" s="7">
         <v>46142</v>
@@ -1119,31 +1179,31 @@
         <v>46142</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="L6" s="6"/>
     </row>
     <row r="7" spans="2:12" ht="26.4" x14ac:dyDescent="0.25">
       <c r="B7" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D7" s="6" t="s">
         <v>24</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="D7" s="6" t="s">
-        <v>26</v>
       </c>
       <c r="E7" s="4" t="s">
         <v>15</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="G7" s="7">
         <v>46135</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="I7" s="7">
         <v>46145</v>
@@ -1152,24 +1212,44 @@
         <v>46145</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="L7" s="6" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="8" spans="2:12" ht="39.6" x14ac:dyDescent="0.25">
+      <c r="B8" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="E8" s="4" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B8" s="2"/>
-      <c r="C8" s="2"/>
-      <c r="D8" s="6"/>
-      <c r="E8" s="4"/>
-      <c r="F8" s="4"/>
-      <c r="G8" s="2"/>
-      <c r="H8" s="2"/>
-      <c r="I8" s="2"/>
+      <c r="F8" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="G8" s="7">
+        <v>46155</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="I8" s="7">
+        <v>46159</v>
+      </c>
       <c r="J8" s="2"/>
-      <c r="K8" s="2"/>
-      <c r="L8" s="6"/>
+      <c r="K8" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="L8" s="6" t="s">
+        <v>37</v>
+      </c>
     </row>
     <row r="9" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B9" s="2"/>
@@ -1488,6 +1568,7 @@
     <mergeCell ref="B1:L1"/>
     <mergeCell ref="B2:L2"/>
   </mergeCells>
+  <phoneticPr fontId="7" type="noConversion"/>
   <printOptions gridLines="1"/>
   <pageMargins left="0.28999999999999998" right="0.27" top="0.48" bottom="0.38" header="0.18" footer="0.17"/>
   <pageSetup scale="90" fitToHeight="3" orientation="landscape" r:id="rId1"/>

</xml_diff>